<commit_message>
ORLANDO-569. Se emparejaron tablas de archivo para importar. Se quitó columna Tipo embalaje.
</commit_message>
<xml_diff>
--- a/src/Files/ImportarMateriales_Consolidado.xlsx
+++ b/src/Files/ImportarMateriales_Consolidado.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25200" windowHeight="12045" activeTab="1"/>
+    <workbookView windowWidth="28125" windowHeight="12375"/>
   </bookViews>
   <sheets>
     <sheet name=" Asignar datos" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="52">
   <si>
     <t>Asignar datos complemento carta porte NODO Materiales</t>
   </si>
@@ -41,7 +41,7 @@
     <t>Clave material peligroso</t>
   </si>
   <si>
-    <t>Tipo embalaje</t>
+    <t>Clave Embalaje</t>
   </si>
   <si>
     <t>Descripción embalaje</t>
@@ -138,6 +138,9 @@
     <t>01010101</t>
   </si>
   <si>
+    <t>KGM</t>
+  </si>
+  <si>
     <t>05</t>
   </si>
   <si>
@@ -176,6 +179,9 @@
     <t>Clave catCartaPorte:c_MaterialPeligroso (catálogo del SAT)</t>
   </si>
   <si>
+    <t>Tipo embalaje</t>
+  </si>
+  <si>
     <t xml:space="preserve">Atributo condicional para precisar la clave del tipo de embalaje que se 
 requiere para transportar el material o residuo peligroso.
 </t>
@@ -209,10 +215,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="178" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="28">
@@ -269,28 +275,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
@@ -299,31 +283,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -338,14 +299,31 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -359,6 +337,29 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
@@ -367,16 +368,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="15"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -392,15 +392,14 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -408,6 +407,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -459,7 +465,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -471,7 +477,133 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -483,55 +615,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -543,37 +627,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -591,55 +645,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -850,15 +856,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -874,30 +871,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
@@ -909,6 +882,17 @@
       </top>
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -939,159 +923,181 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
+      <top/>
+      <bottom style="medium">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
       </top>
       <bottom style="double">
-        <color theme="4"/>
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="22" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1164,13 +1170,10 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1183,11 +1186,14 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1202,54 +1208,54 @@
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="40% - Accent1" xfId="1" builtinId="31"/>
-    <cellStyle name="Comma" xfId="2" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="3" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
-    <cellStyle name="Currency" xfId="5" builtinId="4"/>
-    <cellStyle name="Percent" xfId="6" builtinId="5"/>
-    <cellStyle name="Hyperlink" xfId="7" builtinId="8"/>
-    <cellStyle name="60% - Accent4" xfId="8" builtinId="44"/>
-    <cellStyle name="Followed Hyperlink" xfId="9" builtinId="9"/>
-    <cellStyle name="Check Cell" xfId="10" builtinId="23"/>
-    <cellStyle name="Heading 2" xfId="11" builtinId="17"/>
-    <cellStyle name="Note" xfId="12" builtinId="10"/>
-    <cellStyle name="40% - Accent3" xfId="13" builtinId="39"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11"/>
-    <cellStyle name="40% - Accent2" xfId="15" builtinId="35"/>
-    <cellStyle name="Title" xfId="16" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="17" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="18" builtinId="16"/>
-    <cellStyle name="Heading 3" xfId="19" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="20" builtinId="19"/>
-    <cellStyle name="Input" xfId="21" builtinId="20"/>
-    <cellStyle name="60% - Accent3" xfId="22" builtinId="40"/>
-    <cellStyle name="Good" xfId="23" builtinId="26"/>
-    <cellStyle name="Output" xfId="24" builtinId="21"/>
-    <cellStyle name="20% - Accent1" xfId="25" builtinId="30"/>
-    <cellStyle name="Calculation" xfId="26" builtinId="22"/>
-    <cellStyle name="Linked Cell" xfId="27" builtinId="24"/>
-    <cellStyle name="Total" xfId="28" builtinId="25"/>
-    <cellStyle name="Bad" xfId="29" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="30" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="31" builtinId="29"/>
-    <cellStyle name="20% - Accent5" xfId="32" builtinId="46"/>
-    <cellStyle name="60% - Accent1" xfId="33" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="34" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="35" builtinId="34"/>
-    <cellStyle name="20% - Accent6" xfId="36" builtinId="50"/>
-    <cellStyle name="60% - Accent2" xfId="37" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="38" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="39" builtinId="38"/>
-    <cellStyle name="Accent4" xfId="40" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="41" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="42" builtinId="43"/>
-    <cellStyle name="Accent5" xfId="43" builtinId="45"/>
-    <cellStyle name="40% - Accent5" xfId="44" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="45" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="46" builtinId="49"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
+    <cellStyle name="Título 3" xfId="1" builtinId="18"/>
+    <cellStyle name="Moneda [0]" xfId="2" builtinId="7"/>
+    <cellStyle name="40% - Énfasis1" xfId="3" builtinId="31"/>
+    <cellStyle name="Coma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Moneda" xfId="5" builtinId="4"/>
+    <cellStyle name="Coma" xfId="6" builtinId="3"/>
+    <cellStyle name="Porcentaje" xfId="7" builtinId="5"/>
+    <cellStyle name="Hipervínculo" xfId="8" builtinId="8"/>
+    <cellStyle name="Hipervínculo visitado" xfId="9" builtinId="9"/>
+    <cellStyle name="Salida" xfId="10" builtinId="21"/>
+    <cellStyle name="Nota" xfId="11" builtinId="10"/>
+    <cellStyle name="Título 2" xfId="12" builtinId="17"/>
+    <cellStyle name="Texto de advertencia" xfId="13" builtinId="11"/>
+    <cellStyle name="Título" xfId="14" builtinId="15"/>
+    <cellStyle name="Texto explicativo" xfId="15" builtinId="53"/>
+    <cellStyle name="Título 1" xfId="16" builtinId="16"/>
+    <cellStyle name="Título 4" xfId="17" builtinId="19"/>
+    <cellStyle name="Entrada" xfId="18" builtinId="20"/>
+    <cellStyle name="Cálculo" xfId="19" builtinId="22"/>
+    <cellStyle name="Celda de comprobación" xfId="20" builtinId="23"/>
+    <cellStyle name="Celda vinculada" xfId="21" builtinId="24"/>
+    <cellStyle name="Total" xfId="22" builtinId="25"/>
+    <cellStyle name="Correcto" xfId="23" builtinId="26"/>
+    <cellStyle name="40% - Énfasis5" xfId="24" builtinId="47"/>
+    <cellStyle name="Incorrecto" xfId="25" builtinId="27"/>
+    <cellStyle name="Neutro" xfId="26" builtinId="28"/>
+    <cellStyle name="20% - Énfasis5" xfId="27" builtinId="46"/>
+    <cellStyle name="Énfasis1" xfId="28" builtinId="29"/>
+    <cellStyle name="20% - Énfasis1" xfId="29" builtinId="30"/>
+    <cellStyle name="60% - Énfasis1" xfId="30" builtinId="32"/>
+    <cellStyle name="20% - Énfasis6" xfId="31" builtinId="50"/>
+    <cellStyle name="Énfasis2" xfId="32" builtinId="33"/>
+    <cellStyle name="20% - Énfasis2" xfId="33" builtinId="34"/>
+    <cellStyle name="40% - Énfasis2" xfId="34" builtinId="35"/>
+    <cellStyle name="60% - Énfasis2" xfId="35" builtinId="36"/>
+    <cellStyle name="Énfasis3" xfId="36" builtinId="37"/>
+    <cellStyle name="20% - Énfasis3" xfId="37" builtinId="38"/>
+    <cellStyle name="40% - Énfasis3" xfId="38" builtinId="39"/>
+    <cellStyle name="60% - Énfasis3" xfId="39" builtinId="40"/>
+    <cellStyle name="Énfasis4" xfId="40" builtinId="41"/>
+    <cellStyle name="20% - Énfasis4" xfId="41" builtinId="42"/>
+    <cellStyle name="40% - Énfasis4" xfId="42" builtinId="43"/>
+    <cellStyle name="60% - Énfasis4" xfId="43" builtinId="44"/>
+    <cellStyle name="Énfasis5" xfId="44" builtinId="45"/>
+    <cellStyle name="60% - Énfasis5" xfId="45" builtinId="48"/>
+    <cellStyle name="Énfasis6" xfId="46" builtinId="49"/>
+    <cellStyle name="40% - Énfasis6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Énfasis6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1498,31 +1504,31 @@
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultColWidth="14.4285714285714" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="8.85714285714286" customWidth="1"/>
-    <col min="2" max="2" width="24.4285714285714" customWidth="1"/>
-    <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="11.4285714285714" customWidth="1"/>
-    <col min="5" max="5" width="18.4285714285714" customWidth="1"/>
-    <col min="6" max="6" width="21.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="13.1428571428571" customWidth="1"/>
-    <col min="8" max="8" width="18.8571428571429" customWidth="1"/>
-    <col min="9" max="9" width="12.1428571428571" customWidth="1"/>
-    <col min="10" max="10" width="16.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="74.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="27.1428571428571" customWidth="1"/>
+    <col min="3" max="3" width="38.2857142857143" customWidth="1"/>
+    <col min="4" max="4" width="13.5714285714286" customWidth="1"/>
+    <col min="5" max="5" width="21.2857142857143" customWidth="1"/>
+    <col min="6" max="6" width="24.5714285714286" customWidth="1"/>
+    <col min="7" max="7" width="14.7142857142857" customWidth="1"/>
+    <col min="8" max="8" width="21.8571428571429" customWidth="1"/>
+    <col min="9" max="9" width="5.85714285714286" customWidth="1"/>
+    <col min="10" max="10" width="14.7142857142857" customWidth="1"/>
     <col min="11" max="26" width="10.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.5" customHeight="1" spans="1:26">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="48"/>
       <c r="K1" s="49"/>
       <c r="L1" s="49"/>
@@ -1542,17 +1548,17 @@
       <c r="Z1" s="49"/>
     </row>
     <row r="2" ht="13.5" customHeight="1" spans="1:26">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
       <c r="J2" s="50"/>
       <c r="K2" s="49"/>
       <c r="L2" s="49"/>
@@ -1572,28 +1578,28 @@
       <c r="Z2" s="49"/>
     </row>
     <row r="3" ht="13.5" customHeight="1" spans="1:26">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="45" t="s">
+      <c r="B3" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="45" t="s">
+      <c r="C3" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="45" t="s">
+      <c r="D3" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="45" t="s">
+      <c r="E3" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="45" t="s">
+      <c r="F3" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="45" t="s">
+      <c r="G3" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="45" t="s">
+      <c r="H3" s="31" t="s">
         <v>9</v>
       </c>
       <c r="I3" s="51" t="s">
@@ -15601,7 +15607,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S1000"/>
+  <dimension ref="A1:T1000"/>
   <sheetFormatPr defaultColWidth="14.4285714285714" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="24.4285714285714" customWidth="1"/>
@@ -15610,20 +15616,21 @@
     <col min="4" max="4" width="25.4285714285714" customWidth="1"/>
     <col min="5" max="5" width="39.1428571428571" customWidth="1"/>
     <col min="6" max="6" width="7.71428571428571" customWidth="1"/>
-    <col min="7" max="7" width="8.28571428571429" customWidth="1"/>
-    <col min="8" max="8" width="21.2857142857143" customWidth="1"/>
-    <col min="9" max="9" width="20.7142857142857" customWidth="1"/>
-    <col min="10" max="10" width="19.1428571428571" customWidth="1"/>
-    <col min="11" max="11" width="23.1428571428571" customWidth="1"/>
-    <col min="12" max="12" width="19.2857142857143" customWidth="1"/>
-    <col min="13" max="13" width="22.1428571428571" customWidth="1"/>
-    <col min="14" max="14" width="20.7142857142857" customWidth="1"/>
-    <col min="15" max="15" width="18.7142857142857" customWidth="1"/>
-    <col min="16" max="16" width="20.8571428571429" customWidth="1"/>
-    <col min="17" max="17" width="12.8571428571429" customWidth="1"/>
-    <col min="18" max="18" width="19.2857142857143" customWidth="1"/>
-    <col min="19" max="19" width="12.4285714285714" customWidth="1"/>
-    <col min="20" max="25" width="10.7142857142857" customWidth="1"/>
+    <col min="7" max="7" width="36.1428571428571" customWidth="1"/>
+    <col min="8" max="8" width="27.1428571428571" customWidth="1"/>
+    <col min="9" max="9" width="38.2857142857143" customWidth="1"/>
+    <col min="10" max="10" width="13.5714285714286" customWidth="1"/>
+    <col min="11" max="11" width="21.2857142857143" customWidth="1"/>
+    <col min="12" max="12" width="24.5714285714286" customWidth="1"/>
+    <col min="13" max="13" width="14.7142857142857" customWidth="1"/>
+    <col min="14" max="14" width="21.8571428571429" customWidth="1"/>
+    <col min="15" max="15" width="5.85714285714286" customWidth="1"/>
+    <col min="16" max="16" width="14.7142857142857" customWidth="1"/>
+    <col min="17" max="17" width="20.8571428571429" customWidth="1"/>
+    <col min="18" max="18" width="12.8571428571429" customWidth="1"/>
+    <col min="19" max="19" width="19.2857142857143" customWidth="1"/>
+    <col min="20" max="20" width="12.4285714285714" customWidth="1"/>
+    <col min="21" max="26" width="10.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.5" customHeight="1" spans="1:1">
@@ -15636,7 +15643,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" ht="13.5" customHeight="1" spans="1:17">
+    <row r="3" ht="13.5" customHeight="1" spans="1:18">
       <c r="A3" s="3" t="s">
         <v>14</v>
       </c>
@@ -15662,11 +15669,12 @@
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
       <c r="N3" s="5"/>
-      <c r="O3" s="29"/>
-      <c r="P3" s="30"/>
-      <c r="Q3" s="30"/>
-    </row>
-    <row r="4" ht="13.5" customHeight="1" spans="1:17">
+      <c r="O3" s="5"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="40"/>
+      <c r="R3" s="40"/>
+    </row>
+    <row r="4" ht="13.5" customHeight="1" spans="1:18">
       <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
@@ -15690,11 +15698,12 @@
       <c r="L4" s="10"/>
       <c r="M4" s="10"/>
       <c r="N4" s="10"/>
-      <c r="O4" s="31"/>
-      <c r="P4" s="32"/>
-      <c r="Q4" s="32"/>
-    </row>
-    <row r="5" ht="13.5" customHeight="1" spans="1:15">
+      <c r="O4" s="10"/>
+      <c r="P4" s="30"/>
+      <c r="Q4" s="41"/>
+      <c r="R4" s="41"/>
+    </row>
+    <row r="5" ht="13.5" customHeight="1" spans="1:16">
       <c r="A5" s="6" t="s">
         <v>23</v>
       </c>
@@ -15714,29 +15723,32 @@
       <c r="H5" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="12" t="s">
+      <c r="I5" s="31" t="s">
+        <v>4</v>
+      </c>
+      <c r="J5" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="12" t="s">
+      <c r="K5" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="K5" s="12" t="s">
+      <c r="L5" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="L5" s="12" t="s">
+      <c r="M5" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="M5" s="12" t="s">
+      <c r="N5" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="N5" s="33" t="s">
+      <c r="O5" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="O5" s="34" t="s">
+      <c r="P5" s="33" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" ht="13.5" customHeight="1" spans="1:15">
+    <row r="6" ht="13.5" customHeight="1" spans="1:16">
       <c r="A6" s="6" t="s">
         <v>5</v>
       </c>
@@ -15760,10 +15772,10 @@
         <v>30</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="L6" s="13" t="s">
         <v>32</v>
@@ -15771,26 +15783,29 @@
       <c r="M6" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="N6" s="35">
+      <c r="N6" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="O6" s="34">
         <v>3</v>
       </c>
-      <c r="O6" s="13" t="s">
-        <v>34</v>
+      <c r="P6" s="13" t="s">
+        <v>35</v>
       </c>
     </row>
-    <row r="7" ht="13.5" customHeight="1" spans="1:15">
+    <row r="7" ht="13.5" customHeight="1" spans="1:16">
       <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D7" s="14"/>
       <c r="E7" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G7" s="15"/>
       <c r="H7" s="15"/>
@@ -15799,24 +15814,25 @@
       <c r="K7" s="15"/>
       <c r="L7" s="15"/>
       <c r="M7" s="15"/>
-      <c r="N7" s="36"/>
-      <c r="O7" s="15"/>
-    </row>
-    <row r="8" ht="13.5" customHeight="1" spans="1:15">
+      <c r="N7" s="15"/>
+      <c r="O7" s="35"/>
+      <c r="P7" s="15"/>
+    </row>
+    <row r="8" ht="13.5" customHeight="1" spans="1:16">
       <c r="A8" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G8" s="17"/>
       <c r="H8" s="17"/>
@@ -15825,80 +15841,83 @@
       <c r="K8" s="17"/>
       <c r="L8" s="17"/>
       <c r="M8" s="17"/>
-      <c r="N8" s="37"/>
-      <c r="O8" s="17"/>
-    </row>
-    <row r="9" ht="13.5" customHeight="1" spans="1:19">
+      <c r="N8" s="17"/>
+      <c r="O8" s="36"/>
+      <c r="P8" s="17"/>
+    </row>
+    <row r="9" ht="13.5" customHeight="1" spans="1:20">
       <c r="A9" s="6" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G9" s="19"/>
       <c r="H9" s="20"/>
       <c r="I9" s="20"/>
-      <c r="J9" s="38"/>
-      <c r="K9" s="39"/>
-      <c r="L9" s="39"/>
-      <c r="M9" s="39"/>
-      <c r="N9" s="39"/>
-      <c r="O9" s="39"/>
-      <c r="P9" s="39"/>
-      <c r="Q9" s="39"/>
-      <c r="R9" s="39"/>
-      <c r="S9" s="39"/>
-    </row>
-    <row r="10" ht="13.5" customHeight="1" spans="1:19">
+      <c r="J9" s="20"/>
+      <c r="K9" s="37"/>
+      <c r="L9" s="38"/>
+      <c r="M9" s="38"/>
+      <c r="N9" s="38"/>
+      <c r="O9" s="38"/>
+      <c r="P9" s="38"/>
+      <c r="Q9" s="38"/>
+      <c r="R9" s="38"/>
+      <c r="S9" s="38"/>
+      <c r="T9" s="38"/>
+    </row>
+    <row r="10" ht="13.5" customHeight="1" spans="1:20">
       <c r="A10" s="21" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D10" s="23"/>
       <c r="E10" s="24" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G10" s="25"/>
       <c r="H10" s="26"/>
       <c r="I10" s="26"/>
-      <c r="J10" s="40"/>
+      <c r="J10" s="26"/>
       <c r="K10" s="39"/>
-      <c r="L10" s="39"/>
-      <c r="M10" s="39"/>
-      <c r="N10" s="39"/>
-      <c r="O10" s="39"/>
-      <c r="P10" s="39"/>
-      <c r="Q10" s="39"/>
-      <c r="R10" s="39"/>
-      <c r="S10" s="39"/>
-    </row>
-    <row r="11" ht="59.25" customHeight="1" spans="1:19">
+      <c r="L10" s="38"/>
+      <c r="M10" s="38"/>
+      <c r="N10" s="38"/>
+      <c r="O10" s="38"/>
+      <c r="P10" s="38"/>
+      <c r="Q10" s="38"/>
+      <c r="R10" s="38"/>
+      <c r="S10" s="38"/>
+      <c r="T10" s="38"/>
+    </row>
+    <row r="11" ht="59.25" customHeight="1" spans="1:20">
       <c r="A11" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>20</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D11" s="8"/>
       <c r="E11" s="27" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G11" s="28"/>
       <c r="H11" s="28"/>
@@ -15913,8 +15932,9 @@
       <c r="Q11" s="28"/>
       <c r="R11" s="28"/>
       <c r="S11" s="28"/>
-    </row>
-    <row r="12" ht="45.75" customHeight="1" spans="7:19">
+      <c r="T11" s="28"/>
+    </row>
+    <row r="12" ht="45.75" customHeight="1" spans="7:20">
       <c r="G12" s="28"/>
       <c r="H12" s="28"/>
       <c r="I12" s="28"/>
@@ -15928,8 +15948,9 @@
       <c r="Q12" s="28"/>
       <c r="R12" s="28"/>
       <c r="S12" s="28"/>
-    </row>
-    <row r="13" ht="45.75" customHeight="1" spans="7:19">
+      <c r="T12" s="28"/>
+    </row>
+    <row r="13" ht="45.75" customHeight="1" spans="7:20">
       <c r="G13" s="28"/>
       <c r="H13" s="28"/>
       <c r="I13" s="28"/>
@@ -15943,8 +15964,9 @@
       <c r="Q13" s="28"/>
       <c r="R13" s="28"/>
       <c r="S13" s="28"/>
-    </row>
-    <row r="14" ht="63.75" customHeight="1" spans="7:19">
+      <c r="T13" s="28"/>
+    </row>
+    <row r="14" ht="63.75" customHeight="1" spans="7:20">
       <c r="G14" s="28"/>
       <c r="H14" s="28"/>
       <c r="I14" s="28"/>
@@ -15958,6 +15980,7 @@
       <c r="Q14" s="28"/>
       <c r="R14" s="28"/>
       <c r="S14" s="28"/>
+      <c r="T14" s="28"/>
     </row>
     <row r="15" ht="13.5" customHeight="1"/>
     <row r="16" ht="13.5" customHeight="1"/>
@@ -16950,7 +16973,7 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="D9:D10"/>
-    <mergeCell ref="G9:J10"/>
+    <mergeCell ref="G9:K10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="1" orientation="portrait"/>

</xml_diff>